<commit_message>
liu data 2025 processed
</commit_message>
<xml_diff>
--- a/data/liu/original_data/Linköping 2025.xlsx
+++ b/data/liu/original_data/Linköping 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anngo25\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/liu/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71FF4534-996D-4048-B0F6-65E2034E6449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E92798-3507-5046-8BBE-4501755C0C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="78460" yWindow="1820" windowWidth="31720" windowHeight="20860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Artiklar" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="277">
   <si>
     <t>institution</t>
   </si>
@@ -109,9 +109,6 @@
   </si>
   <si>
     <t>https://www.mdpi.com/2226-4310/12/1/1</t>
-  </si>
-  <si>
-    <t>s42003-024-07448-z</t>
   </si>
   <si>
     <t>Springer Nature</t>
@@ -871,7 +868,7 @@
     <t>978-3-534-64146-8</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>10.1038/s42003-024-07448-z</t>
   </si>
 </sst>
 </file>
@@ -899,6 +896,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1274,12 +1272,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K73"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="7" max="7" width="58.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="58.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6">
+    <row r="1" spans="1:11" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1328,7 +1326,7 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
@@ -1354,7 +1352,7 @@
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
@@ -1380,7 +1378,7 @@
         <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F4" t="s">
         <v>21</v>
@@ -1403,19 +1401,19 @@
         <v>48072</v>
       </c>
       <c r="D5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" t="s">
-        <v>229</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>25</v>
       </c>
-      <c r="G5" t="s">
+      <c r="K5" t="s">
         <v>26</v>
-      </c>
-      <c r="K5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1429,19 +1427,19 @@
         <v>25482</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
       </c>
       <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" t="s">
         <v>29</v>
-      </c>
-      <c r="K6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1455,19 +1453,19 @@
         <v>22799</v>
       </c>
       <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>228</v>
+      </c>
+      <c r="F7" t="s">
         <v>31</v>
       </c>
-      <c r="E7" t="s">
-        <v>229</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>32</v>
       </c>
-      <c r="G7" t="s">
+      <c r="K7" t="s">
         <v>33</v>
-      </c>
-      <c r="K7" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1481,19 +1479,19 @@
         <v>21276</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
       </c>
       <c r="G8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" t="s">
         <v>36</v>
-      </c>
-      <c r="K8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1507,19 +1505,19 @@
         <v>52705</v>
       </c>
       <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F9" t="s">
         <v>38</v>
       </c>
-      <c r="E9" t="s">
-        <v>229</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>39</v>
       </c>
-      <c r="G9" t="s">
+      <c r="K9" t="s">
         <v>40</v>
-      </c>
-      <c r="K9" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1533,19 +1531,19 @@
         <v>25334</v>
       </c>
       <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="E10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="K10" t="s">
         <v>43</v>
-      </c>
-      <c r="K10" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1559,19 +1557,19 @@
         <v>50068</v>
       </c>
       <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s">
+        <v>228</v>
+      </c>
+      <c r="F11" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" t="s">
+        <v>39</v>
+      </c>
+      <c r="K11" t="s">
         <v>45</v>
-      </c>
-      <c r="E11" t="s">
-        <v>229</v>
-      </c>
-      <c r="F11" t="s">
-        <v>39</v>
-      </c>
-      <c r="G11" t="s">
-        <v>40</v>
-      </c>
-      <c r="K11" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1585,19 +1583,19 @@
         <v>23919</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F12" t="s">
         <v>21</v>
       </c>
       <c r="G12" t="s">
+        <v>47</v>
+      </c>
+      <c r="K12" t="s">
         <v>48</v>
-      </c>
-      <c r="K12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1611,19 +1609,19 @@
         <v>10110</v>
       </c>
       <c r="D13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" t="s">
         <v>50</v>
       </c>
-      <c r="E13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>51</v>
       </c>
-      <c r="G13" t="s">
+      <c r="K13" t="s">
         <v>52</v>
-      </c>
-      <c r="K13" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1637,19 +1635,19 @@
         <v>26261</v>
       </c>
       <c r="D14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" t="s">
         <v>54</v>
       </c>
-      <c r="E14" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>55</v>
       </c>
-      <c r="G14" t="s">
+      <c r="K14" t="s">
         <v>56</v>
-      </c>
-      <c r="K14" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1663,19 +1661,19 @@
         <v>22108</v>
       </c>
       <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>228</v>
+      </c>
+      <c r="F15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" t="s">
         <v>58</v>
       </c>
-      <c r="E15" t="s">
-        <v>229</v>
-      </c>
-      <c r="F15" t="s">
-        <v>32</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="K15" t="s">
         <v>59</v>
-      </c>
-      <c r="K15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1689,19 +1687,19 @@
         <v>19444</v>
       </c>
       <c r="D16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s">
+        <v>228</v>
+      </c>
+      <c r="F16" t="s">
         <v>61</v>
       </c>
-      <c r="E16" t="s">
-        <v>229</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>62</v>
       </c>
-      <c r="G16" t="s">
+      <c r="K16" t="s">
         <v>63</v>
-      </c>
-      <c r="K16" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1715,19 +1713,19 @@
         <v>20043</v>
       </c>
       <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" t="s">
         <v>65</v>
       </c>
-      <c r="E17" t="s">
-        <v>117</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>66</v>
       </c>
-      <c r="G17" t="s">
+      <c r="K17" t="s">
         <v>67</v>
-      </c>
-      <c r="K17" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1741,19 +1739,19 @@
         <v>24763</v>
       </c>
       <c r="D18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" t="s">
         <v>69</v>
       </c>
-      <c r="E18" t="s">
-        <v>117</v>
-      </c>
-      <c r="F18" t="s">
-        <v>32</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="K18" t="s">
         <v>70</v>
-      </c>
-      <c r="K18" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1767,19 +1765,19 @@
         <v>28593</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F19" t="s">
         <v>21</v>
       </c>
       <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="K19" t="s">
         <v>73</v>
-      </c>
-      <c r="K19" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1793,19 +1791,19 @@
         <v>25240</v>
       </c>
       <c r="D20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>228</v>
+      </c>
+      <c r="F20" t="s">
         <v>75</v>
       </c>
-      <c r="E20" t="s">
-        <v>229</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>76</v>
       </c>
-      <c r="G20" t="s">
+      <c r="K20" t="s">
         <v>77</v>
-      </c>
-      <c r="K20" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1819,10 +1817,10 @@
         <v>22545</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E21" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F21" t="s">
         <v>21</v>
@@ -1831,7 +1829,7 @@
         <v>22</v>
       </c>
       <c r="K21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1845,19 +1843,19 @@
         <v>34713</v>
       </c>
       <c r="D22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" t="s">
+        <v>116</v>
+      </c>
+      <c r="F22" t="s">
         <v>81</v>
       </c>
-      <c r="E22" t="s">
-        <v>117</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>82</v>
       </c>
-      <c r="G22" t="s">
+      <c r="K22" t="s">
         <v>83</v>
-      </c>
-      <c r="K22" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1871,19 +1869,19 @@
         <v>51824</v>
       </c>
       <c r="D23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" t="s">
+        <v>116</v>
+      </c>
+      <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="E23" t="s">
-        <v>117</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>86</v>
       </c>
-      <c r="G23" t="s">
+      <c r="K23" t="s">
         <v>87</v>
-      </c>
-      <c r="K23" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1897,19 +1895,19 @@
         <v>28633</v>
       </c>
       <c r="D24" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" t="s">
+        <v>228</v>
+      </c>
+      <c r="F24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" t="s">
         <v>89</v>
       </c>
-      <c r="E24" t="s">
-        <v>229</v>
-      </c>
-      <c r="F24" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="K24" t="s">
         <v>90</v>
-      </c>
-      <c r="K24" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1923,19 +1921,19 @@
         <v>47916</v>
       </c>
       <c r="D25" t="s">
+        <v>91</v>
+      </c>
+      <c r="E25" t="s">
+        <v>228</v>
+      </c>
+      <c r="F25" t="s">
+        <v>38</v>
+      </c>
+      <c r="G25" t="s">
+        <v>39</v>
+      </c>
+      <c r="K25" t="s">
         <v>92</v>
-      </c>
-      <c r="E25" t="s">
-        <v>229</v>
-      </c>
-      <c r="F25" t="s">
-        <v>39</v>
-      </c>
-      <c r="G25" t="s">
-        <v>40</v>
-      </c>
-      <c r="K25" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1949,19 +1947,19 @@
         <v>29040</v>
       </c>
       <c r="D26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" t="s">
         <v>94</v>
       </c>
-      <c r="E26" t="s">
-        <v>117</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>95</v>
       </c>
-      <c r="G26" t="s">
+      <c r="K26" t="s">
         <v>96</v>
-      </c>
-      <c r="K26" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1975,19 +1973,19 @@
         <v>52637</v>
       </c>
       <c r="D27" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" t="s">
+        <v>116</v>
+      </c>
+      <c r="F27" t="s">
         <v>98</v>
       </c>
-      <c r="E27" t="s">
-        <v>117</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>99</v>
       </c>
-      <c r="G27" t="s">
+      <c r="K27" t="s">
         <v>100</v>
-      </c>
-      <c r="K27" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2001,19 +1999,19 @@
         <v>16802</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E28" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F28" t="s">
         <v>21</v>
       </c>
       <c r="G28" t="s">
+        <v>102</v>
+      </c>
+      <c r="K28" t="s">
         <v>103</v>
-      </c>
-      <c r="K28" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2027,19 +2025,19 @@
         <v>10784</v>
       </c>
       <c r="D29" t="s">
+        <v>104</v>
+      </c>
+      <c r="E29" t="s">
+        <v>228</v>
+      </c>
+      <c r="F29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G29" t="s">
+        <v>58</v>
+      </c>
+      <c r="K29" t="s">
         <v>105</v>
-      </c>
-      <c r="E29" t="s">
-        <v>229</v>
-      </c>
-      <c r="F29" t="s">
-        <v>32</v>
-      </c>
-      <c r="G29" t="s">
-        <v>59</v>
-      </c>
-      <c r="K29" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2053,19 +2051,19 @@
         <v>9932</v>
       </c>
       <c r="D30" t="s">
+        <v>106</v>
+      </c>
+      <c r="E30" t="s">
+        <v>228</v>
+      </c>
+      <c r="F30" t="s">
         <v>107</v>
       </c>
-      <c r="E30" t="s">
-        <v>229</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>108</v>
       </c>
-      <c r="G30" t="s">
+      <c r="K30" t="s">
         <v>109</v>
-      </c>
-      <c r="K30" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2079,19 +2077,19 @@
         <v>4020</v>
       </c>
       <c r="D31" t="s">
+        <v>110</v>
+      </c>
+      <c r="E31" t="s">
+        <v>228</v>
+      </c>
+      <c r="F31" t="s">
         <v>111</v>
       </c>
-      <c r="E31" t="s">
-        <v>229</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
+        <v>111</v>
+      </c>
+      <c r="K31" t="s">
         <v>112</v>
-      </c>
-      <c r="G31" t="s">
-        <v>112</v>
-      </c>
-      <c r="K31" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2105,19 +2103,19 @@
         <v>18889</v>
       </c>
       <c r="D32" t="s">
+        <v>113</v>
+      </c>
+      <c r="E32" t="s">
+        <v>228</v>
+      </c>
+      <c r="F32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G32" t="s">
+        <v>32</v>
+      </c>
+      <c r="K32" t="s">
         <v>114</v>
-      </c>
-      <c r="E32" t="s">
-        <v>229</v>
-      </c>
-      <c r="F32" t="s">
-        <v>32</v>
-      </c>
-      <c r="G32" t="s">
-        <v>33</v>
-      </c>
-      <c r="K32" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2131,19 +2129,19 @@
         <v>17833</v>
       </c>
       <c r="D33" t="s">
+        <v>115</v>
+      </c>
+      <c r="E33" t="s">
         <v>116</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>117</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>118</v>
       </c>
-      <c r="G33" t="s">
+      <c r="K33" t="s">
         <v>119</v>
-      </c>
-      <c r="K33" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2157,19 +2155,19 @@
         <v>6401</v>
       </c>
       <c r="D34" t="s">
+        <v>120</v>
+      </c>
+      <c r="E34" t="s">
+        <v>116</v>
+      </c>
+      <c r="F34" t="s">
+        <v>31</v>
+      </c>
+      <c r="G34" t="s">
         <v>121</v>
       </c>
-      <c r="E34" t="s">
-        <v>117</v>
-      </c>
-      <c r="F34" t="s">
-        <v>32</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="K34" t="s">
         <v>122</v>
-      </c>
-      <c r="K34" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2183,19 +2181,19 @@
         <v>19315</v>
       </c>
       <c r="D35" t="s">
+        <v>123</v>
+      </c>
+      <c r="E35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F35" t="s">
+        <v>31</v>
+      </c>
+      <c r="G35" t="s">
         <v>124</v>
       </c>
-      <c r="E35" t="s">
-        <v>117</v>
-      </c>
-      <c r="F35" t="s">
-        <v>32</v>
-      </c>
-      <c r="G35" t="s">
+      <c r="K35" t="s">
         <v>125</v>
-      </c>
-      <c r="K35" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2209,19 +2207,19 @@
         <v>23701</v>
       </c>
       <c r="D36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E36" t="s">
+        <v>116</v>
+      </c>
+      <c r="F36" t="s">
+        <v>31</v>
+      </c>
+      <c r="G36" t="s">
         <v>127</v>
       </c>
-      <c r="E36" t="s">
-        <v>117</v>
-      </c>
-      <c r="F36" t="s">
-        <v>32</v>
-      </c>
-      <c r="G36" t="s">
+      <c r="K36" t="s">
         <v>128</v>
-      </c>
-      <c r="K36" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2235,19 +2233,19 @@
         <v>23355</v>
       </c>
       <c r="D37" t="s">
+        <v>129</v>
+      </c>
+      <c r="E37" t="s">
+        <v>228</v>
+      </c>
+      <c r="F37" t="s">
         <v>130</v>
       </c>
-      <c r="E37" t="s">
-        <v>229</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>131</v>
       </c>
-      <c r="G37" t="s">
+      <c r="K37" t="s">
         <v>132</v>
-      </c>
-      <c r="K37" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2261,19 +2259,19 @@
         <v>23362</v>
       </c>
       <c r="D38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E38" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F38" t="s">
         <v>21</v>
       </c>
       <c r="G38" t="s">
+        <v>134</v>
+      </c>
+      <c r="K38" t="s">
         <v>135</v>
-      </c>
-      <c r="K38" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2287,19 +2285,19 @@
         <v>28229</v>
       </c>
       <c r="D39" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F39" t="s">
         <v>21</v>
       </c>
       <c r="G39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2313,19 +2311,19 @@
         <v>33318</v>
       </c>
       <c r="D40" t="s">
+        <v>138</v>
+      </c>
+      <c r="E40" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" t="s">
         <v>139</v>
       </c>
-      <c r="E40" t="s">
-        <v>117</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>140</v>
       </c>
-      <c r="G40" t="s">
+      <c r="K40" t="s">
         <v>141</v>
-      </c>
-      <c r="K40" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2339,19 +2337,19 @@
         <v>23004</v>
       </c>
       <c r="D41" t="s">
+        <v>142</v>
+      </c>
+      <c r="E41" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" t="s">
         <v>143</v>
       </c>
-      <c r="E41" t="s">
-        <v>117</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>144</v>
       </c>
-      <c r="G41" t="s">
+      <c r="K41" t="s">
         <v>145</v>
-      </c>
-      <c r="K41" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2365,19 +2363,19 @@
         <v>35321</v>
       </c>
       <c r="D42" t="s">
+        <v>146</v>
+      </c>
+      <c r="E42" t="s">
+        <v>228</v>
+      </c>
+      <c r="F42" t="s">
         <v>147</v>
       </c>
-      <c r="E42" t="s">
-        <v>229</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>148</v>
       </c>
-      <c r="G42" t="s">
+      <c r="K42" t="s">
         <v>149</v>
-      </c>
-      <c r="K42" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2391,19 +2389,19 @@
         <v>57728</v>
       </c>
       <c r="D43" t="s">
+        <v>150</v>
+      </c>
+      <c r="E43" t="s">
+        <v>116</v>
+      </c>
+      <c r="F43" t="s">
         <v>151</v>
       </c>
-      <c r="E43" t="s">
-        <v>117</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>152</v>
       </c>
-      <c r="G43" t="s">
+      <c r="K43" t="s">
         <v>153</v>
-      </c>
-      <c r="K43" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2417,19 +2415,19 @@
         <v>24905</v>
       </c>
       <c r="D44" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E44" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F44" t="s">
         <v>21</v>
       </c>
       <c r="G44" t="s">
+        <v>155</v>
+      </c>
+      <c r="K44" t="s">
         <v>156</v>
-      </c>
-      <c r="K44" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2443,19 +2441,19 @@
         <v>33312</v>
       </c>
       <c r="D45" t="s">
+        <v>157</v>
+      </c>
+      <c r="E45" t="s">
+        <v>228</v>
+      </c>
+      <c r="F45" t="s">
         <v>158</v>
       </c>
-      <c r="E45" t="s">
-        <v>229</v>
-      </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>159</v>
       </c>
-      <c r="G45" t="s">
+      <c r="K45" t="s">
         <v>160</v>
-      </c>
-      <c r="K45" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2469,19 +2467,19 @@
         <v>12326</v>
       </c>
       <c r="D46" t="s">
+        <v>161</v>
+      </c>
+      <c r="E46" t="s">
+        <v>116</v>
+      </c>
+      <c r="F46" t="s">
         <v>162</v>
       </c>
-      <c r="E46" t="s">
-        <v>117</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>163</v>
       </c>
-      <c r="G46" t="s">
+      <c r="K46" t="s">
         <v>164</v>
-      </c>
-      <c r="K46" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2495,19 +2493,19 @@
         <v>20449</v>
       </c>
       <c r="D47" t="s">
+        <v>165</v>
+      </c>
+      <c r="E47" t="s">
+        <v>228</v>
+      </c>
+      <c r="F47" t="s">
+        <v>31</v>
+      </c>
+      <c r="G47" t="s">
+        <v>32</v>
+      </c>
+      <c r="K47" t="s">
         <v>166</v>
-      </c>
-      <c r="E47" t="s">
-        <v>229</v>
-      </c>
-      <c r="F47" t="s">
-        <v>32</v>
-      </c>
-      <c r="G47" t="s">
-        <v>33</v>
-      </c>
-      <c r="K47" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -2521,19 +2519,19 @@
         <v>21778</v>
       </c>
       <c r="D48" t="s">
+        <v>167</v>
+      </c>
+      <c r="E48" t="s">
+        <v>116</v>
+      </c>
+      <c r="F48" t="s">
         <v>168</v>
       </c>
-      <c r="E48" t="s">
-        <v>117</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>169</v>
       </c>
-      <c r="G48" t="s">
+      <c r="K48" t="s">
         <v>170</v>
-      </c>
-      <c r="K48" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -2547,19 +2545,19 @@
         <v>20299</v>
       </c>
       <c r="D49" t="s">
+        <v>171</v>
+      </c>
+      <c r="E49" t="s">
+        <v>116</v>
+      </c>
+      <c r="F49" t="s">
+        <v>65</v>
+      </c>
+      <c r="G49" t="s">
         <v>172</v>
       </c>
-      <c r="E49" t="s">
-        <v>117</v>
-      </c>
-      <c r="F49" t="s">
-        <v>66</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="K49" t="s">
         <v>173</v>
-      </c>
-      <c r="K49" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -2573,19 +2571,19 @@
         <v>13857</v>
       </c>
       <c r="D50" t="s">
+        <v>174</v>
+      </c>
+      <c r="E50" t="s">
+        <v>228</v>
+      </c>
+      <c r="F50" t="s">
+        <v>158</v>
+      </c>
+      <c r="G50" t="s">
         <v>175</v>
       </c>
-      <c r="E50" t="s">
-        <v>229</v>
-      </c>
-      <c r="F50" t="s">
-        <v>159</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="K50" t="s">
         <v>176</v>
-      </c>
-      <c r="K50" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -2599,19 +2597,19 @@
         <v>33404</v>
       </c>
       <c r="D51" t="s">
+        <v>177</v>
+      </c>
+      <c r="E51" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" t="s">
         <v>178</v>
       </c>
-      <c r="E51" t="s">
-        <v>117</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>179</v>
       </c>
-      <c r="G51" t="s">
+      <c r="K51" t="s">
         <v>180</v>
-      </c>
-      <c r="K51" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -2625,19 +2623,19 @@
         <v>34983</v>
       </c>
       <c r="D52" t="s">
+        <v>181</v>
+      </c>
+      <c r="E52" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" t="s">
         <v>182</v>
       </c>
-      <c r="E52" t="s">
-        <v>117</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>183</v>
       </c>
-      <c r="G52" t="s">
+      <c r="K52" t="s">
         <v>184</v>
-      </c>
-      <c r="K52" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -2651,19 +2649,19 @@
         <v>56455</v>
       </c>
       <c r="D53" t="s">
+        <v>185</v>
+      </c>
+      <c r="E53" t="s">
+        <v>116</v>
+      </c>
+      <c r="F53" t="s">
+        <v>151</v>
+      </c>
+      <c r="G53" t="s">
         <v>186</v>
       </c>
-      <c r="E53" t="s">
-        <v>117</v>
-      </c>
-      <c r="F53" t="s">
-        <v>152</v>
-      </c>
-      <c r="G53" t="s">
+      <c r="K53" t="s">
         <v>187</v>
-      </c>
-      <c r="K53" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -2677,19 +2675,19 @@
         <v>41814</v>
       </c>
       <c r="D54" t="s">
+        <v>188</v>
+      </c>
+      <c r="E54" t="s">
+        <v>116</v>
+      </c>
+      <c r="F54" t="s">
         <v>189</v>
       </c>
-      <c r="E54" t="s">
-        <v>117</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>190</v>
       </c>
-      <c r="G54" t="s">
+      <c r="K54" t="s">
         <v>191</v>
-      </c>
-      <c r="K54" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -2703,19 +2701,19 @@
         <v>24462</v>
       </c>
       <c r="D55" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E55" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F55" t="s">
         <v>21</v>
       </c>
       <c r="G55" t="s">
+        <v>193</v>
+      </c>
+      <c r="K55" t="s">
         <v>194</v>
-      </c>
-      <c r="K55" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -2729,19 +2727,19 @@
         <v>27336</v>
       </c>
       <c r="D56" t="s">
+        <v>195</v>
+      </c>
+      <c r="E56" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" t="s">
         <v>196</v>
       </c>
-      <c r="E56" t="s">
-        <v>117</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
         <v>197</v>
       </c>
-      <c r="G56" t="s">
+      <c r="K56" t="s">
         <v>198</v>
-      </c>
-      <c r="K56" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -2755,19 +2753,19 @@
         <v>39527</v>
       </c>
       <c r="D57" t="s">
+        <v>199</v>
+      </c>
+      <c r="E57" t="s">
+        <v>228</v>
+      </c>
+      <c r="F57" t="s">
+        <v>85</v>
+      </c>
+      <c r="G57" t="s">
         <v>200</v>
       </c>
-      <c r="E57" t="s">
-        <v>229</v>
-      </c>
-      <c r="F57" t="s">
-        <v>86</v>
-      </c>
-      <c r="G57" t="s">
+      <c r="K57" t="s">
         <v>201</v>
-      </c>
-      <c r="K57" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -2781,19 +2779,19 @@
         <v>20911</v>
       </c>
       <c r="D58" t="s">
+        <v>202</v>
+      </c>
+      <c r="E58" t="s">
+        <v>228</v>
+      </c>
+      <c r="F58" t="s">
         <v>203</v>
       </c>
-      <c r="E58" t="s">
-        <v>229</v>
-      </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
         <v>204</v>
       </c>
-      <c r="G58" t="s">
+      <c r="K58" t="s">
         <v>205</v>
-      </c>
-      <c r="K58" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -2807,19 +2805,19 @@
         <v>18838</v>
       </c>
       <c r="D59" t="s">
+        <v>206</v>
+      </c>
+      <c r="E59" t="s">
+        <v>116</v>
+      </c>
+      <c r="F59" t="s">
+        <v>65</v>
+      </c>
+      <c r="G59" t="s">
+        <v>66</v>
+      </c>
+      <c r="K59" t="s">
         <v>207</v>
-      </c>
-      <c r="E59" t="s">
-        <v>117</v>
-      </c>
-      <c r="F59" t="s">
-        <v>66</v>
-      </c>
-      <c r="G59" t="s">
-        <v>67</v>
-      </c>
-      <c r="K59" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -2833,19 +2831,19 @@
         <v>18280</v>
       </c>
       <c r="D60" t="s">
+        <v>208</v>
+      </c>
+      <c r="E60" t="s">
+        <v>228</v>
+      </c>
+      <c r="F60" t="s">
         <v>209</v>
       </c>
-      <c r="E60" t="s">
-        <v>229</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
         <v>210</v>
       </c>
-      <c r="G60" t="s">
+      <c r="K60" t="s">
         <v>211</v>
-      </c>
-      <c r="K60" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -2859,19 +2857,19 @@
         <v>48928</v>
       </c>
       <c r="D61" t="s">
+        <v>212</v>
+      </c>
+      <c r="E61" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" t="s">
         <v>213</v>
       </c>
-      <c r="E61" t="s">
-        <v>117</v>
-      </c>
-      <c r="F61" t="s">
+      <c r="G61" t="s">
         <v>214</v>
       </c>
-      <c r="G61" t="s">
+      <c r="K61" t="s">
         <v>215</v>
-      </c>
-      <c r="K61" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -2885,19 +2883,19 @@
         <v>26323</v>
       </c>
       <c r="D62" t="s">
+        <v>216</v>
+      </c>
+      <c r="E62" t="s">
+        <v>228</v>
+      </c>
+      <c r="F62" t="s">
         <v>217</v>
       </c>
-      <c r="E62" t="s">
-        <v>229</v>
-      </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
         <v>218</v>
       </c>
-      <c r="G62" t="s">
+      <c r="K62" t="s">
         <v>219</v>
-      </c>
-      <c r="K62" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="63" spans="1:11">
@@ -2911,19 +2909,19 @@
         <v>37936</v>
       </c>
       <c r="D63" t="s">
+        <v>220</v>
+      </c>
+      <c r="E63" t="s">
+        <v>116</v>
+      </c>
+      <c r="F63" t="s">
+        <v>182</v>
+      </c>
+      <c r="G63" t="s">
         <v>221</v>
       </c>
-      <c r="E63" t="s">
-        <v>117</v>
-      </c>
-      <c r="F63" t="s">
-        <v>183</v>
-      </c>
-      <c r="G63" t="s">
+      <c r="K63" t="s">
         <v>222</v>
-      </c>
-      <c r="K63" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -2937,19 +2935,19 @@
         <v>50057</v>
       </c>
       <c r="D64" t="s">
+        <v>223</v>
+      </c>
+      <c r="E64" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" t="s">
         <v>224</v>
       </c>
-      <c r="E64" t="s">
-        <v>117</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
         <v>225</v>
       </c>
-      <c r="G64" t="s">
+      <c r="K64" t="s">
         <v>226</v>
-      </c>
-      <c r="K64" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -2963,19 +2961,19 @@
         <v>19715</v>
       </c>
       <c r="D65" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E65" t="s">
+        <v>228</v>
+      </c>
+      <c r="F65" t="s">
+        <v>189</v>
+      </c>
+      <c r="G65" t="s">
         <v>229</v>
       </c>
-      <c r="F65" t="s">
-        <v>190</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="K65" t="s">
         <v>230</v>
-      </c>
-      <c r="K65" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -2989,19 +2987,19 @@
         <v>27120</v>
       </c>
       <c r="D66" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E66" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F66" t="s">
         <v>21</v>
       </c>
       <c r="G66" t="s">
+        <v>232</v>
+      </c>
+      <c r="K66" t="s">
         <v>233</v>
-      </c>
-      <c r="K66" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -3015,19 +3013,19 @@
         <v>1295</v>
       </c>
       <c r="D67" t="s">
+        <v>234</v>
+      </c>
+      <c r="E67" t="s">
+        <v>228</v>
+      </c>
+      <c r="F67" t="s">
         <v>235</v>
       </c>
-      <c r="E67" t="s">
-        <v>229</v>
-      </c>
-      <c r="F67" t="s">
+      <c r="G67" t="s">
         <v>236</v>
       </c>
-      <c r="G67" t="s">
+      <c r="K67" t="s">
         <v>237</v>
-      </c>
-      <c r="K67" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -3041,19 +3039,19 @@
         <v>19439</v>
       </c>
       <c r="D68" t="s">
+        <v>238</v>
+      </c>
+      <c r="E68" t="s">
+        <v>228</v>
+      </c>
+      <c r="F68" t="s">
+        <v>31</v>
+      </c>
+      <c r="G68" t="s">
+        <v>32</v>
+      </c>
+      <c r="K68" t="s">
         <v>239</v>
-      </c>
-      <c r="E68" t="s">
-        <v>229</v>
-      </c>
-      <c r="F68" t="s">
-        <v>32</v>
-      </c>
-      <c r="G68" t="s">
-        <v>33</v>
-      </c>
-      <c r="K68" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -3067,19 +3065,19 @@
         <v>18438</v>
       </c>
       <c r="D69" t="s">
+        <v>240</v>
+      </c>
+      <c r="E69" t="s">
+        <v>228</v>
+      </c>
+      <c r="F69" t="s">
         <v>241</v>
       </c>
-      <c r="E69" t="s">
-        <v>229</v>
-      </c>
-      <c r="F69" t="s">
+      <c r="G69" t="s">
         <v>242</v>
       </c>
-      <c r="G69" t="s">
+      <c r="K69" t="s">
         <v>243</v>
-      </c>
-      <c r="K69" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3093,19 +3091,19 @@
         <v>33856</v>
       </c>
       <c r="D70" t="s">
+        <v>244</v>
+      </c>
+      <c r="E70" t="s">
+        <v>116</v>
+      </c>
+      <c r="F70" t="s">
         <v>245</v>
       </c>
-      <c r="E70" t="s">
-        <v>117</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>246</v>
       </c>
-      <c r="G70" t="s">
+      <c r="K70" t="s">
         <v>247</v>
-      </c>
-      <c r="K70" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -3119,19 +3117,19 @@
         <v>24778</v>
       </c>
       <c r="D71" t="s">
+        <v>248</v>
+      </c>
+      <c r="E71" t="s">
+        <v>116</v>
+      </c>
+      <c r="F71" t="s">
+        <v>31</v>
+      </c>
+      <c r="G71" t="s">
+        <v>42</v>
+      </c>
+      <c r="K71" t="s">
         <v>249</v>
-      </c>
-      <c r="E71" t="s">
-        <v>117</v>
-      </c>
-      <c r="F71" t="s">
-        <v>32</v>
-      </c>
-      <c r="G71" t="s">
-        <v>43</v>
-      </c>
-      <c r="K71" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -3145,19 +3143,19 @@
         <v>40828</v>
       </c>
       <c r="D72" t="s">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>116</v>
+      </c>
+      <c r="F72" t="s">
+        <v>189</v>
+      </c>
+      <c r="G72" t="s">
         <v>251</v>
       </c>
-      <c r="E72" t="s">
-        <v>117</v>
-      </c>
-      <c r="F72" t="s">
-        <v>190</v>
-      </c>
-      <c r="G72" t="s">
+      <c r="K72" t="s">
         <v>252</v>
-      </c>
-      <c r="K72" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3171,19 +3169,19 @@
         <v>25440</v>
       </c>
       <c r="D73" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E73" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F73" t="s">
         <v>21</v>
       </c>
       <c r="G73" t="s">
+        <v>254</v>
+      </c>
+      <c r="K73" t="s">
         <v>255</v>
-      </c>
-      <c r="K73" t="s">
-        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -3196,13 +3194,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95D23D7F-AFED-4151-A314-20E993D1A726}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="93.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="93.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3220,22 +3218,22 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>257</v>
+      </c>
+      <c r="H1" t="s">
         <v>258</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>259</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>260</v>
-      </c>
-      <c r="J1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -3249,19 +3247,19 @@
         <v>134165</v>
       </c>
       <c r="D2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="E2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" t="s">
         <v>263</v>
-      </c>
-      <c r="H2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3275,19 +3273,19 @@
         <v>37076</v>
       </c>
       <c r="D3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E3" t="s">
+        <v>228</v>
+      </c>
+      <c r="F3" t="s">
         <v>265</v>
       </c>
-      <c r="E3" t="s">
-        <v>229</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>266</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>267</v>
-      </c>
-      <c r="H3" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3301,19 +3299,19 @@
         <v>76791</v>
       </c>
       <c r="D4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E4" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" t="s">
         <v>269</v>
       </c>
-      <c r="E4" t="s">
-        <v>229</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>270</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" s="6" t="s">
         <v>271</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -3327,24 +3325,19 @@
         <v>11690</v>
       </c>
       <c r="D5" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F5" t="s">
         <v>273</v>
       </c>
-      <c r="E5" t="s">
-        <v>229</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>274</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>275</v>
-      </c>
-      <c r="H5" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="E11" t="s">
-        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -3353,12 +3346,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x0101005ED58573E86FF944B2D72D3756F3A95B" ma:contentTypeVersion="4" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="950cc0dfaec3a37bd242524d8e992671">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cf08b820-9447-487f-8ef6-1e52edb87de4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="40c3306d27e2406a18572a374cf551a7" ns2:_="">
     <xsd:import namespace="cf08b820-9447-487f-8ef6-1e52edb87de4"/>
@@ -3502,6 +3489,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3512,22 +3505,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBD9F3C9-484A-4CDF-B1AD-46E34198EAA3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="cf08b820-9447-487f-8ef6-1e52edb87de4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D2B8D02-5F2B-46FD-901C-A1760E7FF4B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3545,6 +3522,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBD9F3C9-484A-4CDF-B1AD-46E34198EAA3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="cf08b820-9447-487f-8ef6-1e52edb87de4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{408CED96-6596-48B0-96A7-DBA48BC2B17D}">
   <ds:schemaRefs>

</xml_diff>